<commit_message>
Add import tag mapping plan and refresh the version 3 tester review.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/doc/AbCS_Version3_Release_Tester_Review.xlsx
+++ b/doc/AbCS_Version3_Release_Tester_Review.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Version 3 Plans" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Version 3 Plans'!$A$1:$K$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Version 3 Plans'!$A$1:$K$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -658,7 +658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1819,17 +1819,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Follow-on - Post-v3</t>
+          <t>Follow-on</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Better plot search</t>
+          <t>View-mode field announcements</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Faster search inside long plot summaries on very large libraries.</t>
+          <t>In Book Details view mode, tabbing a field should speak the name and value without JAWS saying edit or read only. Edit mode stays a real edit field.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr"/>
@@ -1837,7 +1837,7 @@
       <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>3-5 days</t>
+          <t>2-4 days</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -1847,12 +1847,12 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Full-text index sync and rebuild add complexity.</t>
+          <t>Must keep real edit widgets in edit mode; a prior attempt that cleared read-only made JAWS say edit.</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
         <is>
-          <t>Post-v3; most useful on very large libraries</t>
+          <t>Anytime / accessibility</t>
         </is>
       </c>
     </row>
@@ -1949,22 +1949,22 @@
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>B01</t>
+          <t>F17</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Follow-on</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Import from other apps</t>
+          <t>Import tag mapping</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Import a library export from another tool (for example Libib or similar CSV formats) with less manual editing.</t>
+          <t>In Preferences Import Settings, choose which audio tags fill book title and author (album vs track title, album artist vs artist). Files still group by album so a multi-part book stays one book. Series from the file name stays an import scenario.</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr"/>
@@ -1972,29 +1972,29 @@
       <c r="G29" s="5" t="inlineStr"/>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>1-2 weeks per format</t>
+          <t>2-3 days</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Third-party export formats change; ongoing maintenance per adapter.</t>
+          <t>Wrong default would change existing imports; grouping must stay on album, not track title.</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>Demand-driven after core waves</t>
+          <t>Anytime / import</t>
         </is>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>B02</t>
+          <t>B01</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -2004,12 +2004,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Saved smart lists</t>
+          <t>Import from other apps</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Save a combination of filters (for example unread sci-fi with a plot) and reuse it with one click.</t>
+          <t>Import a library export from another tool (for example Libib or similar CSV formats) with less manual editing.</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr"/>
@@ -2017,29 +2017,29 @@
       <c r="G30" s="5" t="inlineStr"/>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>1-2 weeks</t>
+          <t>1-2 weeks per format</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Users may confuse saved smart lists with normal collections.</t>
+          <t>Third-party export formats change; ongoing maintenance per adapter.</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>After core filter features land</t>
+          <t>Demand-driven after core waves</t>
         </is>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>B03</t>
+          <t>B02</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -2049,12 +2049,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Reading progress</t>
+          <t>Saved smart lists</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Remember how far you got in a book (not just finished or not). Mainly useful if deeper playback support is added later. Not an in-app player.</t>
+          <t>Save a combination of filters (for example unread sci-fi with a plot) and reuse it with one click.</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr"/>
@@ -2062,29 +2062,29 @@
       <c r="G31" s="5" t="inlineStr"/>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>2-3 weeks+</t>
+          <t>1-2 weeks</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>Conflicts with AbCS focus as a collection manager rather than a player.</t>
+          <t>Users may confuse saved smart lists with normal collections.</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
         <is>
-          <t>Demand-driven; deferred unless strong tester demand</t>
+          <t>After core filter features land</t>
         </is>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>B04</t>
+          <t>B03</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -2094,12 +2094,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Tags on books</t>
+          <t>Reading progress</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Multiple labels per book (for example gift or book club) without changing its collection.</t>
+          <t>Remember how far you got in a book (not just finished or not). Mainly useful if deeper playback support is added later. Not an in-app player.</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr"/>
@@ -2107,29 +2107,29 @@
       <c r="G32" s="5" t="inlineStr"/>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>2-3 weeks</t>
+          <t>2-3 weeks+</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>Overlaps conceptually with Want to Read and collections; needs clear guidance.</t>
+          <t>Conflicts with AbCS focus as a collection manager rather than a player.</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
         <is>
-          <t>Demand-driven backlog</t>
+          <t>Demand-driven; deferred unless strong tester demand</t>
         </is>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>B05</t>
+          <t>B04</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -2139,12 +2139,12 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Check for updates</t>
+          <t>Tags on books</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Help menu option to see if a newer AbCS version is available and open the download page. No silent install.</t>
+          <t>Multiple labels per book (for example gift or book club) without changing its collection.</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr"/>
@@ -2152,44 +2152,44 @@
       <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>2-3 days</t>
+          <t>2-3 weeks</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Offline users see nothing; no telemetry in v1.</t>
+          <t>Overlaps conceptually with Want to Read and collections; needs clear guidance.</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
         <is>
-          <t>Anytime; good small release win</t>
+          <t>Demand-driven backlog</t>
         </is>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>M01</t>
+          <t>B05</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Maintenance - not user-facing</t>
+          <t>Backlog</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>CI / test hardening</t>
+          <t>Check for updates</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Strengthen automated regression testing for version 3 waves. Supports safer development. Not a user-visible feature.</t>
+          <t>Help menu option to see if a newer AbCS version is available and open the download page. No silent install.</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr"/>
@@ -2197,7 +2197,7 @@
       <c r="G34" s="5" t="inlineStr"/>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>1-2 days setup + ongoing</t>
+          <t>2-3 days</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
@@ -2207,19 +2207,19 @@
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure work; does not change app features for end users.</t>
+          <t>Offline users see nothing; no telemetry in v1.</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>Between waves; early in the version 3 cycle</t>
+          <t>Anytime; good small release win</t>
         </is>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>M02</t>
+          <t>M01</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -2229,12 +2229,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Dead-code cleanup</t>
+          <t>CI / test hardening</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Periodic cleanup of unused code to keep the project easier to maintain. Not a user-visible feature.</t>
+          <t>Strengthen automated regression testing for version 3 waves. Supports safer development. Not a user-visible feature.</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr"/>
@@ -2242,27 +2242,72 @@
       <c r="G35" s="5" t="inlineStr"/>
       <c r="H35" s="5" t="inlineStr">
         <is>
+          <t>1-2 days setup + ongoing</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>Infrastructure work; does not change app features for end users.</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>Between waves; early in the version 3 cycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance - not user-facing</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Dead-code cleanup</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Periodic cleanup of unused code to keep the project easier to maintain. Not a user-visible feature.</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
           <t>0.5-1 day per pass</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr">
+      <c r="J36" s="5" t="inlineStr">
         <is>
           <t>Only removes confirmed unused code after tests pass.</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr">
+      <c r="K36" s="5" t="inlineStr">
         <is>
           <t>Between waves or before release tags</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K35"/>
+  <autoFilter ref="A1:K36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>